<commit_message>
docs: add student Chau Chi Cuong SE180687 to report, slide, and excel
</commit_message>
<xml_diff>
--- a/AI2108_Group08_SE180687_ChauChiCuong/Ai_Audit_Log_Group08_SE180687.xlsx
+++ b/AI2108_Group08_SE180687_ChauChiCuong/Ai_Audit_Log_Group08_SE180687.xlsx
@@ -1156,7 +1156,7 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Ghép 4 bảng NTSB mà không làm nở số dòng</t>
+          <t>Ghép 4 bảng NTSB (events, aircraft, injury, crew) mà không làm nở số dòng do va chạm nhiều máy bay/phi công.</t>
         </is>
       </c>
       <c r="E5" s="19" t="inlineStr">
@@ -1166,17 +1166,17 @@
       </c>
       <c r="F5" s="19" t="inlineStr">
         <is>
-          <t>AI đề xuất lệnh INNER JOIN đơn giản nối trực tiếp 4 bảng.</t>
+          <t>AI đề xuất lệnh INNER JOIN đơn giản nối trực tiếp 4 bảng theo ev_id.</t>
         </is>
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Critical Thinking: JOIN đơn giản làm tăng từ 57k lên 78k (bùng nổ cartesian). Contextualization: Mỗi sự kiện chỉ 1 dòng. Creative Synthesis: Viết CTE dùng MAX()/FIRST() theo ev_id. Decision Ownership: Giữ chuẩn 57,260 dòng.</t>
+          <t>Critical Thinking: JOIN đơn giản làm số dòng tăng vọt từ 57k lên 78k (bùng nổ cartesian). Contextualization: Mỗi sự kiện chỉ được có đúng 1 dòng đại diện. Creative Synthesis: Tự viết CTE gom nhóm MAX()/FIRST() theo ev_id. Decision Ownership: Dùng CTE gom nhóm để bảng hợp nhất giữ chuẩn 57,260 dòng.</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>report/table_q2_ac_agg.csv</t>
+          <t>report/table_q2_ac_agg.csv + code trong 03_sql_analysis.py</t>
         </is>
       </c>
     </row>
@@ -1196,27 +1196,27 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>Cột inj_tot_f có nhiều ô trống (NULL)</t>
+          <t>Cột inj_tot_f có nhiều ô trống (NULL) trong cơ sở dữ liệu NTSB Access.</t>
         </is>
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>inj_tot_f bị thiếu giá trị, nên dropna hay fill 0?</t>
+          <t>Cột inj_tot_f bị thiếu giá trị, nên xử lý dropna hay fill 0 trong pandas?</t>
         </is>
       </c>
       <c r="F6" s="19" t="inlineStr">
         <is>
-          <t>AI gợi ý dùng dropna(subset=['inj_tot_f']).</t>
+          <t>AI gợi ý sử dụng df.dropna(subset=['inj_tot_f']) để đảm bảo sạch nhãn.</t>
         </is>
       </c>
       <c r="G6" s="19" t="inlineStr">
         <is>
-          <t>Critical Thinking: ẢO GIÁC PHÁT HIỆN. Contextualization: codman.pdf mục 4.2 quy định ô trống ở tai nạn đóng hồ sơ là 0 người chết. Creative Synthesis: Điền 0. Decision Ownership: Bảo toàn 18.2% tỷ lệ tử vong cơ sở.</t>
+          <t>Critical Thinking: HALLUCINATION/ERROR DETECTED. Contextualization: Đối chiếu cẩm nang NTSB codman.pdf, ở tai nạn máy bay tư nhân đã đóng hồ sơ, ô trống nghĩa là 0 nạn nhân chết. Creative Synthesis: Quy đổi NULL thành 0. Decision Ownership: Giữ lại hơn 6,000 dòng không tử vong, bảo toàn tỷ lệ nhãn 18.2%.</t>
         </is>
       </c>
       <c r="H6" s="19" t="inlineStr">
         <is>
-          <t>codman.pdf mục 4.2</t>
+          <t>Trích dẫn Mục 4.2 trong tài liệu NTSB codman.pdf</t>
         </is>
       </c>
     </row>
@@ -1236,27 +1236,27 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Nhận diện drone trong NTSB</t>
+          <t>Nhận diện phương tiện bay không người lái (UAS / drone) trong kho dữ liệu NTSB.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>NTSB phân loại drone bằng mã nào trong acft_category?</t>
+          <t>Cơ sở dữ liệu NTSB phân loại drone bằng mã nào trong cột acft_category?</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>AI khẳng định NTSB dùng mã 'DRONE' từ 1990.</t>
+          <t>AI khẳng định NTSB luôn dùng mã 'DRONE' trong cột acft_category từ năm 1990 đến nay.</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Critical Thinking: ẢO GIÁC PHÁT HIỆN. Contextualization: Mã 'DRONE' không tồn tại. Creative Synthesis: Mã 'UAS' có từ 2018, trước đó dùng 'UNK'/tên hãng. Decision Ownership: Xây dựng bộ lọc regex kết hợp.</t>
+          <t>Critical Thinking: HALLUCINATION DETECTED. Contextualization: Kiểm tra thực tế NTSB không có mã 'DRONE'. Creative Synthesis: NTSB chỉ bắt đầu dùng 'UAS' từ 2018; trước đó sự cố drone ghi nhận ở 'UNK' hoặc tên hãng (DJI, Autel). Decision Ownership: Xây dựng bộ lọc regex kết hợp acft_category và tên nhà sản xuất.</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>SELECT DISTINCT acft_category</t>
+          <t>Kết quả truy vấn SELECT DISTINCT acft_category FROM aircraft</t>
         </is>
       </c>
     </row>
@@ -1276,27 +1276,27 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Chọn đặc trưng không rò rỉ dữ liệu</t>
+          <t>Lựa chọn các cột đặc trưng để dự báo mức độ nghiêm trọng mà không gây rò rỉ dữ liệu.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Đặc trưng nào trong bảng events nên đưa vào mô hình?</t>
+          <t>Liệt kê các đặc trưng quan trọng nhất trong bảng events để đưa vào mô hình học máy?</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>AI đề xuất cả số xe cứu hỏa và nguyên nhân điều tra kết luận.</t>
+          <t>AI đề xuất đưa vào cả số xe cứu hỏa huy động và nguyên nhân điều tra kết luận.</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>Critical Thinking: RÒ RỈ DỮ LIỆU. Contextualization: Biến cứu hỏa chỉ có sau tai nạn. Creative Synthesis: Chỉ giữ biến môi trường, phương tiện, phi công trước bay. Decision Ownership: Loại bỏ toàn bộ biến hậu kỳ.</t>
+          <t>Critical Thinking: RÒ RỈ DỮ LIỆU (Target Leakage). Contextualization: Số xe cứu hỏa và nguyên nhân điều tra chỉ có sau khi tai nạn kết thúc. Creative Synthesis: Chỉ giữ lại các đặc trưng môi trường (thời tiết, ánh sáng), phương tiện và phi công quan sát được trước chuyến bay. Decision Ownership: Loại bỏ toàn bộ biến hậu kỳ.</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>report/table_features.csv</t>
+          <t>Bảng danh mục đặc trưng trong report/table_features.csv</t>
         </is>
       </c>
     </row>
@@ -1316,27 +1316,27 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Giờ bay phi công khuyết 14.6%</t>
+          <t>Cột tổng giờ bay của phi công (pilot_tot_hrs) bị khuyết 14.6%.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Nên điền khuyết giờ bay bằng mean hay median?</t>
+          <t>Nên điền khuyết giờ bay phi công bằng mean toàn bộ hay median?</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>AI đề xuất dùng mean toàn bộ.</t>
+          <t>AI đề xuất dùng df['pilot_tot_hrs'].fillna(df['pilot_tot_hrs'].mean()).</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Critical Thinking: Giờ bay phân phối lệch phải mạnh. Contextualization: Part 121 khác xa Part 91. Creative Synthesis: Dùng Median có điều kiện theo far_part. Decision Ownership: Tránh sai lệch phân khúc.</t>
+          <t>Critical Thinking: Giờ bay phân phối lệch phải (skewed) rất mạnh, mean sẽ bị kéo lệch bởi phi công 30,000h. Contextualization: Phi công thương mại Part 121 có giờ bay khác xa phi công tư nhân Part 91. Creative Synthesis: Dùng Conditional Median Imputation theo far_part. Decision Ownership: Giữ vững tính đại diện của từng phân khúc bay.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>report/table_describe_raw.csv</t>
+          <t>Bảng phân phối giờ bay trong report/table_describe_raw.csv</t>
         </is>
       </c>
     </row>
@@ -1356,27 +1356,27 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Chia tập dữ liệu chuỗi tai nạn</t>
+          <t>Cách chia tập huấn luyện và kiểm thử cho bài toán chuỗi dữ liệu tai nạn.</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>Nên dùng train_test_split ngẫu nhiên không?</t>
+          <t>Nên dùng train_test_split ngẫu nhiên của scikit-learn với test_size=0.2 không?</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>AI gợi ý train_test_split ngẫu nhiên.</t>
+          <t>AI gợi ý dùng train_test_split(test_size=0.2, random_state=42).</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Critical Thinking: Rò rỉ tương lai vào quá khứ. Contextualization: Thực tế dự báo tương lai từ quá khứ. Creative Synthesis: Chia Train (1990-2018), Test (2019-2024), UAS holdout. Decision Ownership: Tuân thủ Temporal Split.</t>
+          <t>Critical Thinking: Chia ngẫu nhiên gây rò rỉ tương lai vào quá khứ. Contextualization: Mô hình thực tế phải dự báo tai nạn trong tương lai dựa trên dữ liệu quá khứ. Creative Synthesis: Chia theo mốc thời gian: Train (1990-2018) và Test (2019-2024), tách riêng drone làm tập đổi miền. Decision Ownership: Tuân thủ giao thức Temporal Split khoa học.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>manifest.json</t>
+          <t>Tệp manifest.json ghi nhận cấu trúc chia tập</t>
         </is>
       </c>
     </row>
@@ -1604,22 +1604,22 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>AI khuyên dropna(inj_tot_f)</t>
+          <t>AI khuyên dropna(subset=['inj_tot_f'])</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>NULL ở sự cố đóng hồ sơ là 0 người chết</t>
+          <t>NULL ở NTSB đối với sự cố tư nhân đóng hồ sơ tương ứng 0 người tử vong, không phải thiếu dữ liệu</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>codman.pdf mục 4.2</t>
+          <t>Đối chiếu cẩm nang NTSB codman.pdf mục 4.2</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Quy đổi NULL về 0, giữ đủ 57,260 dòng</t>
+          <t>Quy đổi NULL về 0, bảo toàn nguyên vẹn 57,260 dòng</t>
         </is>
       </c>
     </row>
@@ -1631,27 +1631,27 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Fabrication / Fact Error</t>
+          <t>Fabrication / Fact</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Mã 'DRONE' có từ 1990</t>
+          <t>AI khẳng định có mã 'DRONE' từ 1990</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Mã 'DRONE' không tồn tại, chỉ có 'UAS' từ 2018</t>
+          <t>Mã 'DRONE' không tồn tại; mã 'UAS' chỉ xuất hiện từ 2018</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>SELECT DISTINCT acft_category</t>
+          <t>Chạy SELECT DISTINCT acft_category trong DuckDB</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Tự viết regex acft_category='UAS' và hãng DJI/Autel</t>
+          <t>Tự tạo bộ lọc regex kết hợp acft_category='UAS' và từ khóa hãng DJI/Autel</t>
         </is>
       </c>
     </row>
@@ -1668,22 +1668,22 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>INNER JOIN trực tiếp 4 bảng</t>
+          <t>AI đề xuất INNER JOIN trực tiếp 4 bảng</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Làm nở số dòng từ 57k lên 78k</t>
+          <t>Làm số dòng tăng từ 57k lên 78k do va chạm nhiều máy bay/nhiều phi công</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>COUNT(*) sau khi JOIN</t>
+          <t>Kiểm tra COUNT(*) sau khi JOIN</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Viết CTE dùng MAX()/FIRST() theo ev_id</t>
+          <t>Viết CTE dùng MAX()/FIRST() gom nhóm về từng ev_id duy nhất</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS (6/6 core prompts)</t>
         </is>
       </c>
       <c r="D14" s="12" t="n"/>
@@ -2156,7 +2156,7 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PASS (All 4 stages covered)</t>
         </is>
       </c>
       <c r="D15" s="12" t="n"/>

</xml_diff>